<commit_message>
allowing excel tabs to have shorter names
</commit_message>
<xml_diff>
--- a/GC2301_BUILDER.xlsx
+++ b/GC2301_BUILDER.xlsx
@@ -8,36 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\TFL_SHELLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E8F4F84-5FBE-40C1-A068-5994B91F55E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D840DF91-DA4C-4C1D-86EA-BFE4E44802BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13749" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13749" tabRatio="1000" firstSheet="9" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TABLE 99" sheetId="34" r:id="rId1"/>
-    <sheet name="TABLE 99__COLUMNS" sheetId="33" r:id="rId2"/>
-    <sheet name="LISTING 1" sheetId="27" r:id="rId3"/>
-    <sheet name="LISTING 1__COLUMNS" sheetId="28" r:id="rId4"/>
+    <sheet name="T 99" sheetId="34" r:id="rId1"/>
+    <sheet name="T 99__COLUMNS" sheetId="33" r:id="rId2"/>
+    <sheet name="L 1" sheetId="27" r:id="rId3"/>
+    <sheet name="L 1__COLUMNS" sheetId="28" r:id="rId4"/>
     <sheet name="DICTIONARY" sheetId="7" r:id="rId5"/>
-    <sheet name="TABLE 14.1.1.1" sheetId="25" r:id="rId6"/>
-    <sheet name="TABLE 14.1.1.1__COLUMNS" sheetId="26" r:id="rId7"/>
-    <sheet name="TABLE 1" sheetId="1" r:id="rId8"/>
-    <sheet name="TABLE 1__COLUMNS" sheetId="2" r:id="rId9"/>
-    <sheet name="TABLE 2" sheetId="10" r:id="rId10"/>
-    <sheet name="TABLE 2__COLUMNS" sheetId="11" r:id="rId11"/>
-    <sheet name="TABLE 3" sheetId="5" r:id="rId12"/>
-    <sheet name="TABLE 3__COLUMNS" sheetId="6" r:id="rId13"/>
-    <sheet name="TABLE 4" sheetId="8" r:id="rId14"/>
-    <sheet name="TABLE 4__COLUMNS" sheetId="9" r:id="rId15"/>
-    <sheet name="TABLE 5" sheetId="12" r:id="rId16"/>
-    <sheet name="TABLE 5__COLUMNS" sheetId="13" r:id="rId17"/>
-    <sheet name="TABLE 6" sheetId="18" r:id="rId18"/>
-    <sheet name="TABLE 6__COLUMNS" sheetId="19" r:id="rId19"/>
-    <sheet name="TABLE 7" sheetId="20" r:id="rId20"/>
-    <sheet name="FIG_1" sheetId="22" r:id="rId21"/>
-    <sheet name="FIG_2" sheetId="23" r:id="rId22"/>
-    <sheet name="FIG_3" sheetId="24" r:id="rId23"/>
-    <sheet name="FIG_4" sheetId="29" r:id="rId24"/>
-    <sheet name="TABLE 7__COLUMNS" sheetId="21" r:id="rId25"/>
+    <sheet name="T 14.1.1.1" sheetId="25" r:id="rId6"/>
+    <sheet name="T 14.1.1.1__COLUMNS" sheetId="26" r:id="rId7"/>
+    <sheet name="T 1" sheetId="1" r:id="rId8"/>
+    <sheet name="T 1__COLUMNS" sheetId="2" r:id="rId9"/>
+    <sheet name="T 2" sheetId="10" r:id="rId10"/>
+    <sheet name="T 2__COLUMNS" sheetId="11" r:id="rId11"/>
+    <sheet name="T 3" sheetId="5" r:id="rId12"/>
+    <sheet name="T 3__COL" sheetId="6" r:id="rId13"/>
+    <sheet name="T 4" sheetId="8" r:id="rId14"/>
+    <sheet name="T 4__C" sheetId="9" r:id="rId15"/>
+    <sheet name="T 5" sheetId="12" r:id="rId16"/>
+    <sheet name="T 5__COLUMNS" sheetId="13" r:id="rId17"/>
+    <sheet name="T 6" sheetId="18" r:id="rId18"/>
+    <sheet name="T 6__COLUMNS" sheetId="19" r:id="rId19"/>
+    <sheet name="T 7" sheetId="20" r:id="rId20"/>
+    <sheet name="T 7__COLUMNS" sheetId="21" r:id="rId21"/>
+    <sheet name="FIG_1" sheetId="22" r:id="rId22"/>
+    <sheet name="FIG_2" sheetId="23" r:id="rId23"/>
+    <sheet name="FIG_3" sheetId="24" r:id="rId24"/>
+    <sheet name="FIG_4" sheetId="29" r:id="rId25"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -4808,1012 +4808,6 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4928F083-95D6-446F-B559-DEE7105C03C2}">
-  <dimension ref="A1:C18"/>
-  <sheetFormatPr defaultRowHeight="15.05"/>
-  <cols>
-    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="29"/>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="29"/>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>153</v>
-      </c>
-      <c r="C3" s="29"/>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="C4" s="29"/>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="29"/>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" s="29"/>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="C7" s="29"/>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" s="31">
-        <v>24</v>
-      </c>
-      <c r="C8" s="29"/>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="31" t="s">
-        <v>157</v>
-      </c>
-      <c r="C9" s="29"/>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="31">
-        <v>0.2</v>
-      </c>
-      <c r="C10" s="29"/>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="B11" s="31">
-        <v>12345</v>
-      </c>
-      <c r="C11" s="29"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="B12" s="32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="27" t="s">
-        <v>161</v>
-      </c>
-      <c r="B13" s="32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="B14" s="32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="B15" s="32">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="B17" s="32">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>167</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE8B490-2B59-40B2-A541-295526A51BDB}">
-  <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15.05"/>
-  <cols>
-    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="29"/>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="29"/>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="C3" s="29"/>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="C4" s="29"/>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="29"/>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" s="29"/>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="C7" s="29"/>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" s="31">
-        <v>24</v>
-      </c>
-      <c r="C8" s="29"/>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="31" t="s">
-        <v>157</v>
-      </c>
-      <c r="C9" s="29"/>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="31">
-        <v>0.2</v>
-      </c>
-      <c r="C10" s="29"/>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="B11" s="31">
-        <v>12345</v>
-      </c>
-      <c r="C11" s="29"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="B12" s="32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="27" t="s">
-        <v>161</v>
-      </c>
-      <c r="B13" s="32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="B14" s="32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="B15" s="32">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="B17" s="32">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>171</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
-        <v>172</v>
-      </c>
-      <c r="B20" s="32" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>173</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
-        <v>174</v>
-      </c>
-      <c r="B22" s="32">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" t="s">
-        <v>176</v>
-      </c>
-      <c r="B23" s="32">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
-        <v>177</v>
-      </c>
-      <c r="B24" s="32">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" t="s">
-        <v>178</v>
-      </c>
-      <c r="B25" s="32">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D40E88A0-2D4A-4482-87C1-7D8FECBED8F0}">
-  <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultRowHeight="15.05"/>
-  <cols>
-    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="29"/>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="E2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="C3" s="29"/>
-      <c r="E3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>180</v>
-      </c>
-      <c r="C4" s="29"/>
-      <c r="E4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="E5" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="C6" s="29"/>
-      <c r="E6" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="C7" s="29"/>
-      <c r="E7" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="29"/>
-      <c r="E8" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="29"/>
-      <c r="E9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="29"/>
-      <c r="E10" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="B11" s="31">
-        <v>12345</v>
-      </c>
-      <c r="C11" s="29"/>
-      <c r="E11" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="E12" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="27" t="s">
-        <v>161</v>
-      </c>
-      <c r="E13" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="E14" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="E15" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="E16" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="E17" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="E18" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>171</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>195</v>
-      </c>
-      <c r="E19" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>172</v>
-      </c>
-      <c r="B20" s="32" t="s">
-        <v>193</v>
-      </c>
-      <c r="E20" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>173</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>194</v>
-      </c>
-      <c r="E21" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>174</v>
-      </c>
-      <c r="B22" s="32">
-        <v>0.6</v>
-      </c>
-      <c r="E22" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
-        <v>176</v>
-      </c>
-      <c r="B23" s="32">
-        <v>10</v>
-      </c>
-      <c r="E23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" t="s">
-        <v>177</v>
-      </c>
-      <c r="B24" s="32">
-        <v>6</v>
-      </c>
-      <c r="E24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" t="s">
-        <v>178</v>
-      </c>
-      <c r="B25" s="32">
-        <v>0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>181</v>
-      </c>
-      <c r="B26" s="32" t="s">
-        <v>182</v>
-      </c>
-      <c r="E26" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>183</v>
-      </c>
-      <c r="B27" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="E27" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" t="s">
-        <v>184</v>
-      </c>
-      <c r="B28" s="32" t="s">
-        <v>185</v>
-      </c>
-      <c r="E28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D4E71C5-0BEA-4A11-9A48-8D675CA18E83}">
-  <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultRowHeight="15.05"/>
-  <cols>
-    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="29" t="s">
-        <v>143</v>
-      </c>
-      <c r="B1" s="31" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="29"/>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="29" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2" s="29"/>
-      <c r="E2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="30" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="C3" s="29"/>
-      <c r="E3" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="30" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>233</v>
-      </c>
-      <c r="C4" s="29"/>
-      <c r="E4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="E5" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="C6" s="29"/>
-      <c r="E6" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="C7" s="29"/>
-      <c r="E7" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="29"/>
-      <c r="E8" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="29"/>
-      <c r="E9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="29"/>
-      <c r="E10" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="B11" s="31">
-        <v>12345</v>
-      </c>
-      <c r="C11" s="29"/>
-      <c r="E11" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="E12" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="27" t="s">
-        <v>161</v>
-      </c>
-      <c r="E13" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="30" t="s">
-        <v>162</v>
-      </c>
-      <c r="E14" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="E15" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="E16" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="E17" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="E18" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>171</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>195</v>
-      </c>
-      <c r="E19" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>172</v>
-      </c>
-      <c r="B20" s="32" t="s">
-        <v>193</v>
-      </c>
-      <c r="E20" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>173</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>194</v>
-      </c>
-      <c r="E21" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>174</v>
-      </c>
-      <c r="B22" s="32">
-        <v>0.6</v>
-      </c>
-      <c r="E22" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
-        <v>176</v>
-      </c>
-      <c r="B23" s="32">
-        <v>10</v>
-      </c>
-      <c r="E23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" t="s">
-        <v>177</v>
-      </c>
-      <c r="B24" s="32">
-        <v>6</v>
-      </c>
-      <c r="E24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" t="s">
-        <v>178</v>
-      </c>
-      <c r="B25" s="32">
-        <v>0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" t="s">
-        <v>181</v>
-      </c>
-      <c r="B26" s="32" t="s">
-        <v>182</v>
-      </c>
-      <c r="E26" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" t="s">
-        <v>183</v>
-      </c>
-      <c r="B27" s="32" t="s">
-        <v>237</v>
-      </c>
-      <c r="E27" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" t="s">
-        <v>184</v>
-      </c>
-      <c r="B28" s="32" t="s">
-        <v>236</v>
-      </c>
-      <c r="E28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{949963F2-1424-438A-8E26-4E7A3C4F92E3}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15.05"/>
@@ -6007,6 +5001,1012 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4928F083-95D6-446F-B559-DEE7105C03C2}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="15.05"/>
+  <cols>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" s="29"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="29"/>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>153</v>
+      </c>
+      <c r="C3" s="29"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" s="29"/>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="29"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="29"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="29"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="31">
+        <v>24</v>
+      </c>
+      <c r="C8" s="29"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="29"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="31">
+        <v>0.2</v>
+      </c>
+      <c r="C10" s="29"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="31">
+        <v>12345</v>
+      </c>
+      <c r="C11" s="29"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="32">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="B17" s="32">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFE8B490-2B59-40B2-A541-295526A51BDB}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="15.05"/>
+  <cols>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" s="29"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="29"/>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="C3" s="29"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="C4" s="29"/>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="29"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="29"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="29"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="31">
+        <v>24</v>
+      </c>
+      <c r="C8" s="29"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="29"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="31">
+        <v>0.2</v>
+      </c>
+      <c r="C10" s="29"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="31">
+        <v>12345</v>
+      </c>
+      <c r="C11" s="29"/>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B13" s="32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" s="32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="32">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="B17" s="32">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="32">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="32">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>178</v>
+      </c>
+      <c r="B25" s="32">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D40E88A0-2D4A-4482-87C1-7D8FECBED8F0}">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="15.05"/>
+  <cols>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" s="29"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="E2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>180</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="E4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="E5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="E6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="E7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="31"/>
+      <c r="C8" s="29"/>
+      <c r="E8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="31"/>
+      <c r="C9" s="29"/>
+      <c r="E9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="31"/>
+      <c r="C10" s="29"/>
+      <c r="E10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="31">
+        <v>12345</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="E11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="E12" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="E13" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="E15" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="E16" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="E17" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="E18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="E19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="E21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="32">
+        <v>0.6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="32">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="32">
+        <v>6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>178</v>
+      </c>
+      <c r="B25" s="32">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>181</v>
+      </c>
+      <c r="B26" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="E26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>183</v>
+      </c>
+      <c r="B27" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="E27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>184</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="E28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D4E71C5-0BEA-4A11-9A48-8D675CA18E83}">
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="15.05"/>
+  <cols>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.88671875" style="32" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" s="29"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="29"/>
+      <c r="E2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="C3" s="29"/>
+      <c r="E3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="30" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="29"/>
+      <c r="E4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="29"/>
+      <c r="E5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="C6" s="29"/>
+      <c r="E6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="C7" s="29"/>
+      <c r="E7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="31"/>
+      <c r="C8" s="29"/>
+      <c r="E8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="31"/>
+      <c r="C9" s="29"/>
+      <c r="E9" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B10" s="31"/>
+      <c r="C10" s="29"/>
+      <c r="E10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="B11" s="31">
+        <v>12345</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="E11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="E12" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="E13" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="E15" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="E16" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="E17" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="E18" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="E19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="E21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="32">
+        <v>0.6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="32">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="32">
+        <v>6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>178</v>
+      </c>
+      <c r="B25" s="32">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>181</v>
+      </c>
+      <c r="B26" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="E26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>183</v>
+      </c>
+      <c r="B27" s="32" t="s">
+        <v>237</v>
+      </c>
+      <c r="E27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>184</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>236</v>
+      </c>
+      <c r="E28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>